<commit_message>
Kit Advogados: título das abas em linha mesclada (20 planilhas regeradas); imagens do site para o kit
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0146uBo6FVJ2cyEehyP8rK61
</commit_message>
<xml_diff>
--- a/projetos/gestao-ia-planilhas/produto/kit-advogados/01-agenda-de-prazos.xlsx
+++ b/projetos/gestao-ia-planilhas/produto/kit-advogados/01-agenda-de-prazos.xlsx
@@ -240,7 +240,9 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -937,7 +939,7 @@
     <col width="10" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="5">
         <f>Config!$B$4&amp;" · Painel de prazos · "&amp;TEXT(Config!$B$5,"dd/mm/yyyy")</f>
         <v/>
@@ -2166,7 +2168,7 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
-  <mergeCells count="33">
+  <mergeCells count="34">
     <mergeCell ref="A48:B48"/>
     <mergeCell ref="A30:B30"/>
     <mergeCell ref="A49:B49"/>
@@ -2195,6 +2197,7 @@
     <mergeCell ref="I4:J4"/>
     <mergeCell ref="A29:B29"/>
     <mergeCell ref="A43:B43"/>
+    <mergeCell ref="A1:L1"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="A44:B44"/>
     <mergeCell ref="K4:L4"/>
@@ -2243,7 +2246,7 @@
     <col width="4" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Configurações</t>
@@ -2477,8 +2480,9 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2505,7 +2509,7 @@
     <col hidden="1" width="6" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Prazos</t>
@@ -11727,7 +11731,8 @@
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
   <autoFilter ref="A4:I404"/>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <conditionalFormatting sqref="A5:I404">

</xml_diff>